<commit_message>
funciona bien, pero hay códigos que no están
</commit_message>
<xml_diff>
--- a/codigos/codigos_ropa.xlsx
+++ b/codigos/codigos_ropa.xlsx
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E109"/>
+  <dimension ref="A1:F109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>Repuesto</t>
+          <t>Descripcion</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -435,6 +435,11 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>Articulo</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Codigos</t>
         </is>
       </c>
     </row>
@@ -458,6 +463,11 @@
       <c r="E2" t="n">
         <v>1</v>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>130.00001</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -479,6 +489,11 @@
       <c r="E3" t="n">
         <v>1</v>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>130.00001</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -500,6 +515,11 @@
       <c r="E4" t="n">
         <v>2</v>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>130.00002</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -521,6 +541,11 @@
       <c r="E5" t="n">
         <v>2</v>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>130.00002</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -542,6 +567,11 @@
       <c r="E6" t="n">
         <v>3</v>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>130.00003</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -563,6 +593,11 @@
       <c r="E7" t="n">
         <v>4</v>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>130.00004</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -584,6 +619,11 @@
       <c r="E8" t="n">
         <v>5</v>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>130.00005</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -605,6 +645,11 @@
       <c r="E9" t="n">
         <v>5</v>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>130.00005</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -626,6 +671,11 @@
       <c r="E10" t="n">
         <v>6</v>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>130.00006</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -647,6 +697,11 @@
       <c r="E11" t="n">
         <v>6</v>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>130.00006</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -668,6 +723,11 @@
       <c r="E12" t="n">
         <v>7</v>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>130.00007</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -689,6 +749,11 @@
       <c r="E13" t="n">
         <v>8</v>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>130.00008</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -710,6 +775,11 @@
       <c r="E14" t="n">
         <v>8</v>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>130.00008</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -731,6 +801,11 @@
       <c r="E15" t="n">
         <v>9</v>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>130.00009</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -752,6 +827,11 @@
       <c r="E16" t="n">
         <v>11</v>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>130.00011</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -773,6 +853,11 @@
       <c r="E17" t="n">
         <v>12</v>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>130.00012</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -794,6 +879,11 @@
       <c r="E18" t="n">
         <v>14</v>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>130.00014</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -815,6 +905,11 @@
       <c r="E19" t="n">
         <v>15</v>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>130.00015</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -836,6 +931,11 @@
       <c r="E20" t="n">
         <v>16</v>
       </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>130.00016</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -857,6 +957,11 @@
       <c r="E21" t="n">
         <v>17</v>
       </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>130.00017</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -878,6 +983,11 @@
       <c r="E22" t="n">
         <v>18</v>
       </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>130.00018</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -899,6 +1009,11 @@
       <c r="E23" t="n">
         <v>19</v>
       </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>130.00019</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -920,6 +1035,11 @@
       <c r="E24" t="n">
         <v>21</v>
       </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>130.00021</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -941,6 +1061,11 @@
       <c r="E25" t="n">
         <v>21</v>
       </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>130.00021</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -962,6 +1087,11 @@
       <c r="E26" t="n">
         <v>22</v>
       </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>130.00022</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -983,6 +1113,11 @@
       <c r="E27" t="n">
         <v>23</v>
       </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>130.00023</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1004,6 +1139,11 @@
       <c r="E28" t="n">
         <v>23</v>
       </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>130.00023</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1025,6 +1165,11 @@
       <c r="E29" t="n">
         <v>24</v>
       </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>130.00024</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1046,6 +1191,11 @@
       <c r="E30" t="n">
         <v>25</v>
       </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>130.00025</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1067,6 +1217,11 @@
       <c r="E31" t="n">
         <v>26</v>
       </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>130.00026</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1088,6 +1243,11 @@
       <c r="E32" t="n">
         <v>26</v>
       </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>130.00026</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1109,6 +1269,11 @@
       <c r="E33" t="n">
         <v>27</v>
       </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>130.00027</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1130,6 +1295,11 @@
       <c r="E34" t="n">
         <v>27</v>
       </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>130.00027</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1151,6 +1321,11 @@
       <c r="E35" t="n">
         <v>28</v>
       </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>130.00028</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1172,6 +1347,11 @@
       <c r="E36" t="n">
         <v>28</v>
       </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>130.00028</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1193,6 +1373,11 @@
       <c r="E37" t="n">
         <v>29</v>
       </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>130.00029</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1214,6 +1399,11 @@
       <c r="E38" t="n">
         <v>29</v>
       </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>130.00029</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1235,6 +1425,11 @@
       <c r="E39" t="n">
         <v>44</v>
       </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>130.00044</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1256,6 +1451,11 @@
       <c r="E40" t="n">
         <v>51</v>
       </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>130.00051</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1277,6 +1477,11 @@
       <c r="E41" t="n">
         <v>57</v>
       </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>130.00057</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1298,6 +1503,11 @@
       <c r="E42" t="n">
         <v>59</v>
       </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>130.00059</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1319,6 +1529,11 @@
       <c r="E43" t="n">
         <v>62</v>
       </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>130.00062</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1340,6 +1555,11 @@
       <c r="E44" t="n">
         <v>63</v>
       </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>130.00063</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1361,6 +1581,11 @@
       <c r="E45" t="n">
         <v>64</v>
       </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>130.00064</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1382,6 +1607,11 @@
       <c r="E46" t="n">
         <v>65</v>
       </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>130.00065</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1403,6 +1633,11 @@
       <c r="E47" t="n">
         <v>76</v>
       </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>130.00076</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1424,6 +1659,11 @@
       <c r="E48" t="n">
         <v>77</v>
       </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>130.00077</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1445,6 +1685,11 @@
       <c r="E49" t="n">
         <v>78</v>
       </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>130.00078</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1466,6 +1711,11 @@
       <c r="E50" t="n">
         <v>79</v>
       </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>130.00079</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1487,6 +1737,11 @@
       <c r="E51" t="n">
         <v>81</v>
       </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>130.00081</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1508,6 +1763,11 @@
       <c r="E52" t="n">
         <v>82</v>
       </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>130.00082</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1529,6 +1789,11 @@
       <c r="E53" t="n">
         <v>85</v>
       </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>130.00085</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1550,6 +1815,11 @@
       <c r="E54" t="n">
         <v>88</v>
       </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>130.00088</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1571,6 +1841,11 @@
       <c r="E55" t="n">
         <v>122</v>
       </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>130.00122</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1592,6 +1867,11 @@
       <c r="E56" t="n">
         <v>125</v>
       </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>130.00125</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1613,6 +1893,11 @@
       <c r="E57" t="n">
         <v>201</v>
       </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>130.00201</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -1634,6 +1919,11 @@
       <c r="E58" t="n">
         <v>202</v>
       </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>130.00202</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1655,6 +1945,11 @@
       <c r="E59" t="n">
         <v>203</v>
       </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>130.00203</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -1676,6 +1971,11 @@
       <c r="E60" t="n">
         <v>204</v>
       </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>130.00204</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -1697,6 +1997,11 @@
       <c r="E61" t="n">
         <v>205</v>
       </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>130.00205</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -1718,6 +2023,11 @@
       <c r="E62" t="n">
         <v>206</v>
       </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>130.00206</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -1739,6 +2049,11 @@
       <c r="E63" t="n">
         <v>207</v>
       </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>130.00207</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -1760,6 +2075,11 @@
       <c r="E64" t="n">
         <v>208</v>
       </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>130.00208</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -1781,6 +2101,11 @@
       <c r="E65" t="n">
         <v>209</v>
       </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>130.00209</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -1802,6 +2127,11 @@
       <c r="E66" t="n">
         <v>211</v>
       </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>130.00211</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -1823,6 +2153,11 @@
       <c r="E67" t="n">
         <v>212</v>
       </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>130.00212</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -1844,6 +2179,11 @@
       <c r="E68" t="n">
         <v>213</v>
       </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>130.00213</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -1865,6 +2205,11 @@
       <c r="E69" t="n">
         <v>221</v>
       </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>130.00221</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -1886,6 +2231,11 @@
       <c r="E70" t="n">
         <v>222</v>
       </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>130.00222</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -1907,6 +2257,11 @@
       <c r="E71" t="n">
         <v>223</v>
       </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>130.00223</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -1928,6 +2283,11 @@
       <c r="E72" t="n">
         <v>224</v>
       </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>130.00224</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -1949,6 +2309,11 @@
       <c r="E73" t="n">
         <v>225</v>
       </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>130.00225</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -1970,6 +2335,11 @@
       <c r="E74" t="n">
         <v>226</v>
       </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>130.00226</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -1991,6 +2361,11 @@
       <c r="E75" t="n">
         <v>227</v>
       </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>130.00227</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -2012,6 +2387,11 @@
       <c r="E76" t="n">
         <v>228</v>
       </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>130.00228</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -2033,6 +2413,11 @@
       <c r="E77" t="n">
         <v>229</v>
       </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>130.00229</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -2054,6 +2439,11 @@
       <c r="E78" t="n">
         <v>232</v>
       </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>130.00232</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -2075,6 +2465,11 @@
       <c r="E79" t="n">
         <v>233</v>
       </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>130.00233</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -2096,6 +2491,11 @@
       <c r="E80" t="n">
         <v>234</v>
       </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>130.00234</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -2117,6 +2517,11 @@
       <c r="E81" t="n">
         <v>252</v>
       </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>130.00252</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -2138,6 +2543,11 @@
       <c r="E82" t="n">
         <v>253</v>
       </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>130.00253</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -2159,6 +2569,11 @@
       <c r="E83" t="n">
         <v>254</v>
       </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>130.00254</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -2180,6 +2595,11 @@
       <c r="E84" t="n">
         <v>255</v>
       </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>130.00255</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -2201,6 +2621,11 @@
       <c r="E85" t="n">
         <v>261</v>
       </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>130.00261</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -2222,6 +2647,11 @@
       <c r="E86" t="n">
         <v>262</v>
       </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>130.00262</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -2243,6 +2673,11 @@
       <c r="E87" t="n">
         <v>263</v>
       </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>130.00263</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -2264,6 +2699,11 @@
       <c r="E88" t="n">
         <v>264</v>
       </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>130.00264</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -2285,6 +2725,11 @@
       <c r="E89" t="n">
         <v>265</v>
       </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>130.00265</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -2306,6 +2751,11 @@
       <c r="E90" t="n">
         <v>266</v>
       </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>130.00266</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -2327,6 +2777,11 @@
       <c r="E91" t="n">
         <v>267</v>
       </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>130.00267</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -2348,6 +2803,11 @@
       <c r="E92" t="n">
         <v>268</v>
       </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>130.00268</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -2369,6 +2829,11 @@
       <c r="E93" t="n">
         <v>271</v>
       </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>130.00271</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -2390,6 +2855,11 @@
       <c r="E94" t="n">
         <v>272</v>
       </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>130.00272</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -2411,6 +2881,11 @@
       <c r="E95" t="n">
         <v>273</v>
       </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>130.00273</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -2432,6 +2907,11 @@
       <c r="E96" t="n">
         <v>274</v>
       </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>130.00274</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -2453,6 +2933,11 @@
       <c r="E97" t="n">
         <v>275</v>
       </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>130.00275</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -2474,6 +2959,11 @@
       <c r="E98" t="n">
         <v>276</v>
       </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>130.00276</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -2495,6 +2985,11 @@
       <c r="E99" t="n">
         <v>277</v>
       </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>130.00277</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -2516,6 +3011,11 @@
       <c r="E100" t="n">
         <v>278</v>
       </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>130.00278</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -2537,6 +3037,11 @@
       <c r="E101" t="n">
         <v>281</v>
       </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>130.00281</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -2558,6 +3063,11 @@
       <c r="E102" t="n">
         <v>282</v>
       </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>130.00282</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -2579,6 +3089,11 @@
       <c r="E103" t="n">
         <v>283</v>
       </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>130.00283</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -2600,6 +3115,11 @@
       <c r="E104" t="n">
         <v>284</v>
       </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>130.00284</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -2621,6 +3141,11 @@
       <c r="E105" t="n">
         <v>285</v>
       </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>130.00285</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -2642,6 +3167,11 @@
       <c r="E106" t="n">
         <v>286</v>
       </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>130.00286</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -2663,6 +3193,11 @@
       <c r="E107" t="n">
         <v>287</v>
       </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>130.00287</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -2684,6 +3219,11 @@
       <c r="E108" t="n">
         <v>288</v>
       </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>130.00288</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -2704,6 +3244,11 @@
       </c>
       <c r="E109" t="n">
         <v>289</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>130.00289</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ahora tambien puede formatear los pedidos pendientes y mejorado el CLI
</commit_message>
<xml_diff>
--- a/codigos/codigos_ropa.xlsx
+++ b/codigos/codigos_ropa.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="227">
   <si>
     <t>Descripcion</t>
   </si>
@@ -34,327 +34,333 @@
     <t>PANTALON DE TRABAJO N°38 VERDE OLIVA</t>
   </si>
   <si>
+    <t>PANTALON DE TRABAJO N°40 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>PANTALON DE TRABAJO N°42 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>PANTALON DE TRABAJO N°44 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>PANTALON DE TRABAJO N°46 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>PANTALON DE TRABAJO N°48 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>PANTALON DE TRABAJO N°50 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>PANTALON DE TRABAJO N°52 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>PANTALON DE TRABAJO N°54 VERDE OLIVA</t>
+  </si>
+  <si>
     <t>PANTALON DE TRABAJO N°56 VERDE OLIVA</t>
   </si>
   <si>
-    <t>PANTALON DE TRABAJO N°40 VERDE OLIVA</t>
+    <t>PANTALON DE TRABAJO N°58 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>PANTALON DE TRABAJO N°60 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>PANTALON DE TRABAJO N°64 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>PANTALON DE TRABAJO N°66 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>CAMISA DE TRABAJO N°38 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>CAMISA DE TRABAJO N°40 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>CAMISA DE TRABAJO N°42 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>CAMISA DE TRABAJO N°44 VERDE OLIVA</t>
   </si>
   <si>
     <t>CAMISA DE TRABAJO N°46 VERDE OLIVA</t>
   </si>
   <si>
-    <t>PANTALON DE TRABAJO N°42 VERDE OLIVA</t>
-  </si>
-  <si>
-    <t>PANTALON DE TRABAJO N°44 VERDE OLIVA</t>
-  </si>
-  <si>
-    <t>PANTALON DE TRABAJO N°46 VERDE OLIVA</t>
+    <t>CAMISA DE TRABAJO N°48 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>CAMISA DE TRABAJO N°50 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>CAMISA DE TRABAJO N°52 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>CAMISA DE TRABAJO N°54 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>CAMISA DE TRABAJO N°56 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>CAMISA DE TRABAJO N°58 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>CAMISA DE TRABAJO N°60 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>CAMISA DE TRABAJO N°62 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>CAMISA DE TRABAJO N°64 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>CAMISA ANTIACIDA AZUL N°40</t>
   </si>
   <si>
     <t>CAMISA ANTIACIDA AZUL N°50</t>
   </si>
   <si>
-    <t>PANTALON DE TRABAJO N°48 VERDE OLIVA</t>
+    <t>CAMISA ANTIACIDA AZUL N°52</t>
+  </si>
+  <si>
+    <t>BOTIN DE TRABAJO N°39</t>
+  </si>
+  <si>
+    <t>BOTIN DE TRABAJO N°40</t>
+  </si>
+  <si>
+    <t>BOTIN DE TRABAJO N°41</t>
   </si>
   <si>
     <t>BOTIN DE TRABAJO N°42</t>
   </si>
   <si>
-    <t>PANTALON DE TRABAJO N°50 VERDE OLIVA</t>
-  </si>
-  <si>
-    <t>PANTALON DE TRABAJO N°52 VERDE OLIVA</t>
+    <t>BOTIN DE TRABAJO N°43</t>
+  </si>
+  <si>
+    <t>BOTIN DE TRABAJO N°44</t>
+  </si>
+  <si>
+    <t>BOTIN DE TRABAJO N°45</t>
+  </si>
+  <si>
+    <t>BOTIN DE TRABAJO N°46</t>
+  </si>
+  <si>
+    <t>BOTIN DE TRABAJO N°47</t>
+  </si>
+  <si>
+    <t>BOTA DE LLUVIA N°41</t>
+  </si>
+  <si>
+    <t>BOTA DE LLUVIA N°40</t>
+  </si>
+  <si>
+    <t>BOTA DE LLUVIA N°42</t>
+  </si>
+  <si>
+    <t>BOTA DE LLUVIA N°43</t>
   </si>
   <si>
     <t>BOTA DE LLUVIA N°44</t>
   </si>
   <si>
-    <t>PANTALON DE TRABAJO N°54 VERDE OLIVA</t>
-  </si>
-  <si>
-    <t>PANTALON DE TRABAJO N°58 VERDE OLIVA</t>
-  </si>
-  <si>
-    <t>PANTALON DE TRABAJO N°60 VERDE OLIVA</t>
-  </si>
-  <si>
-    <t>PANTALON DE TRABAJO N°64 VERDE OLIVA</t>
-  </si>
-  <si>
-    <t>PANTALON DE TRABAJO N°66 VERDE OLIVA</t>
-  </si>
-  <si>
-    <t>CAMISA DE TRABAJO N°38 VERDE OLIVA</t>
-  </si>
-  <si>
-    <t>CAMISA DE TRABAJO N°40 VERDE OLIVA</t>
-  </si>
-  <si>
-    <t>CAMISA DE TRABAJO N°42 VERDE OLIVA</t>
-  </si>
-  <si>
-    <t>CAMISA DE TRABAJO N°44 VERDE OLIVA</t>
+    <t>BOTA DE LLUVIA N°45</t>
+  </si>
+  <si>
+    <t>BOTA DE LLUVIA N°38</t>
+  </si>
+  <si>
+    <t>BOTIN DE TRABAJO N°35</t>
+  </si>
+  <si>
+    <t>BOTA DE LLUVIA N°39</t>
+  </si>
+  <si>
+    <t>CAMISA DE TRABAJO Nº68 VERDE OLIVA</t>
+  </si>
+  <si>
+    <t>BOTA DE LLUVIA N°46</t>
+  </si>
+  <si>
+    <t>CAMISA CHOFER CELESTE TALLE 36</t>
+  </si>
+  <si>
+    <t>CAMISA CHOFER CELESTE TALLE 38</t>
+  </si>
+  <si>
+    <t>CAMISA CHOFER CELESTE TALLE 40</t>
+  </si>
+  <si>
+    <t>CAMISA CHOFER CELESTE TALLE 42</t>
+  </si>
+  <si>
+    <t>CAMISA CHOFER CELESTE TALLE 44</t>
+  </si>
+  <si>
+    <t>CAMISA CHOFER CELESTE TALLE 46</t>
+  </si>
+  <si>
+    <t>CAMISA CHOFER CELESTE TALLE 48</t>
+  </si>
+  <si>
+    <t>CAMISA CHOFER CELESTE TALLE 50</t>
+  </si>
+  <si>
+    <t>CAMISA CHOFER CELESTE TALLE 52</t>
   </si>
   <si>
     <t>CAMISA CHOFER CELESTE TALLE 54</t>
   </si>
   <si>
-    <t>CAMISA DE TRABAJO N°48 VERDE OLIVA</t>
-  </si>
-  <si>
-    <t>CAMISA DE TRABAJO N°50 VERDE OLIVA</t>
+    <t>CAMISA CHOFER CELESTE TALLE 56</t>
+  </si>
+  <si>
+    <t>CAMISA CHOFER CELESTE TALLE 58</t>
+  </si>
+  <si>
+    <t>CAMISA CHOFER CELESTE TALLE 60</t>
+  </si>
+  <si>
+    <t>CAMISA INSPECTOR BLANCA TALLE 36</t>
+  </si>
+  <si>
+    <t>CAMISA INSPECTOR BLANCA TALLE 38</t>
+  </si>
+  <si>
+    <t>CAMISA INSPECTOR BLANCA TALLE 40</t>
+  </si>
+  <si>
+    <t>CAMISA INSPECTOR BLANCA TALLE 42</t>
+  </si>
+  <si>
+    <t>CAMISA INSPECTOR BLANCA TALLE 44</t>
+  </si>
+  <si>
+    <t>CAMISA INSPECTOR BLANCA TALLE 46</t>
+  </si>
+  <si>
+    <t>CAMISA INSPECTOR BLANCA TALLE 48</t>
+  </si>
+  <si>
+    <t>CAMISA INSPECTOR BLANCA TALLE 50</t>
+  </si>
+  <si>
+    <t>CAMISA INSPECTOR BLANCA TALLE 52</t>
   </si>
   <si>
     <t>CAMISA INSPECTOR BLANCA TALLE 54</t>
   </si>
   <si>
-    <t>CAMISA DE TRABAJO N°52 VERDE OLIVA</t>
-  </si>
-  <si>
-    <t>CAMISA DE TRABAJO N°54 VERDE OLIVA</t>
-  </si>
-  <si>
-    <t>CAMISA DE TRABAJO N°56 VERDE OLIVA</t>
+    <t>CAMISA INSPECTOR BLANCA TALLE 58</t>
+  </si>
+  <si>
+    <t>CAMISA INSPECTOR BLANCA TALLE 60</t>
+  </si>
+  <si>
+    <t>CAMISA INSPECTOR BLANCA TALLE 62</t>
+  </si>
+  <si>
+    <t>CAMISA CHOFER MUJER CELESTE TALLE 38</t>
+  </si>
+  <si>
+    <t>CAMISA CHOFER MUJER CELESTE TALLE 40</t>
+  </si>
+  <si>
+    <t>CAMISA CHOFER MUJER CELESTE TALLE 42</t>
+  </si>
+  <si>
+    <t>CAMISA CHOFER MUJER CELESTE TALLE 44</t>
   </si>
   <si>
     <t>CHALECO POLAR NEGRO TALLE S</t>
   </si>
   <si>
-    <t>CAMISA DE TRABAJO N°58 VERDE OLIVA</t>
+    <t>CHALECO POLAR NEGRO TALLE M</t>
+  </si>
+  <si>
+    <t>CHALECO POLAR NEGRO TALLE L</t>
+  </si>
+  <si>
+    <t>CHALECO POLAR NEGRO TALLE XL</t>
+  </si>
+  <si>
+    <t>CHALECO POLAR NEGRO TALLE XXL</t>
+  </si>
+  <si>
+    <t>CHALECO POLAR NEGRO TALLE XXXL</t>
+  </si>
+  <si>
+    <t>CHALECO POLAR NEGRO TALLE 4XL</t>
+  </si>
+  <si>
+    <t>CHALECO POLAR NEGRO TALLE 5XL</t>
+  </si>
+  <si>
+    <t>CHALECO POLAR NEGRO TALLE 6XL</t>
   </si>
   <si>
     <t>CAMPERA INSPECCION NEGRA TALLE S</t>
   </si>
   <si>
-    <t>CAMISA DE TRABAJO N°60 VERDE OLIVA</t>
+    <t>CAMPERA INSPECCION NEGRA TALLE M</t>
+  </si>
+  <si>
+    <t>CAMPERA INSPECCION NEGRA TALLE L</t>
+  </si>
+  <si>
+    <t>CAMPERA INSPECCION NEGRA TALLE XL</t>
+  </si>
+  <si>
+    <t>CAMPERA INSPECCION NEGRA TALLE XXL</t>
+  </si>
+  <si>
+    <t>CAMPERA INSPECCION NEGRA TALLE XXXL</t>
+  </si>
+  <si>
+    <t>CAMPERA INSPECCION NEGRA TALLE 4XL</t>
+  </si>
+  <si>
+    <t>CAMPERA INSPECCION NEGRA TALLE 5XL</t>
+  </si>
+  <si>
+    <t>CAMPERA INSPECCION NEGRA TALLE 6XL</t>
   </si>
   <si>
     <t>CAMPERA CHOFER AZUL TALLE S</t>
   </si>
   <si>
-    <t>CAMISA DE TRABAJO N°62 VERDE OLIVA</t>
+    <t>CAMPERA CHOFER AZUL TALLE M</t>
+  </si>
+  <si>
+    <t>CAMPERA CHOFER AZUL TALLE L</t>
+  </si>
+  <si>
+    <t>CAMPERA CHOFER AZUL TALLE XL</t>
+  </si>
+  <si>
+    <t>CAMPERA CHOFER AZUL TALLE XXL</t>
+  </si>
+  <si>
+    <t>CAMPERA CHOFER AZUL TALLE XXXL</t>
+  </si>
+  <si>
+    <t>CAMPERA CHOFER AZUL TALLE 4XL</t>
+  </si>
+  <si>
+    <t>CAMPERA CHOFER AZUL TALLE 5XL</t>
+  </si>
+  <si>
+    <t>CAMPERA CHOFER AZUL TALLE 6XL</t>
+  </si>
+  <si>
+    <t>CAMPERA CHOFER AZUL TALLE 7XL</t>
   </si>
   <si>
     <t>CAMPERA CHOFER AZUL TALLE XS</t>
   </si>
   <si>
-    <t>CAMISA DE TRABAJO N°64 VERDE OLIVA</t>
-  </si>
-  <si>
-    <t>CAMISA ANTIACIDA AZUL N°40</t>
-  </si>
-  <si>
-    <t>CAMISA ANTIACIDA AZUL N°52</t>
-  </si>
-  <si>
-    <t>BOTIN DE TRABAJO N°39</t>
-  </si>
-  <si>
-    <t>BOTIN DE TRABAJO N°41</t>
-  </si>
-  <si>
-    <t>BOTIN DE TRABAJO N°44</t>
-  </si>
-  <si>
-    <t>BOTIN DE TRABAJO N°45</t>
-  </si>
-  <si>
-    <t>BOTIN DE TRABAJO N°46</t>
-  </si>
-  <si>
-    <t>BOTIN DE TRABAJO N°47</t>
-  </si>
-  <si>
-    <t>BOTA DE LLUVIA N°41</t>
-  </si>
-  <si>
-    <t>BOTA DE LLUVIA N°40</t>
-  </si>
-  <si>
-    <t>BOTA DE LLUVIA N°42</t>
-  </si>
-  <si>
-    <t>BOTA DE LLUVIA N°43</t>
-  </si>
-  <si>
-    <t>BOTA DE LLUVIA N°45</t>
-  </si>
-  <si>
-    <t>BOTA DE LLUVIA N°38</t>
-  </si>
-  <si>
-    <t>BOTIN DE TRABAJO N°35</t>
-  </si>
-  <si>
-    <t>BOTA DE LLUVIA N°39</t>
-  </si>
-  <si>
-    <t>CAMISA DE TRABAJO Nº68 VERDE OLIVA</t>
-  </si>
-  <si>
-    <t>BOTA DE LLUVIA N°46</t>
-  </si>
-  <si>
-    <t>CAMISA CHOFER CELESTE TALLE 36</t>
-  </si>
-  <si>
-    <t>CAMISA CHOFER CELESTE TALLE 38</t>
-  </si>
-  <si>
-    <t>CAMISA CHOFER CELESTE TALLE 40</t>
-  </si>
-  <si>
-    <t>CAMISA CHOFER CELESTE TALLE 42</t>
-  </si>
-  <si>
-    <t>CAMISA CHOFER CELESTE TALLE 44</t>
-  </si>
-  <si>
-    <t>CAMISA CHOFER CELESTE TALLE 46</t>
-  </si>
-  <si>
-    <t>CAMISA CHOFER CELESTE TALLE 48</t>
-  </si>
-  <si>
-    <t>CAMISA CHOFER CELESTE TALLE 50</t>
-  </si>
-  <si>
-    <t>CAMISA CHOFER CELESTE TALLE 52</t>
-  </si>
-  <si>
-    <t>CAMISA CHOFER CELESTE TALLE 56</t>
-  </si>
-  <si>
-    <t>CAMISA CHOFER CELESTE TALLE 58</t>
-  </si>
-  <si>
-    <t>CAMISA CHOFER CELESTE TALLE 60</t>
-  </si>
-  <si>
-    <t>CAMISA INSPECTOR BLANCA TALLE 36</t>
-  </si>
-  <si>
-    <t>CAMISA INSPECTOR BLANCA TALLE 38</t>
-  </si>
-  <si>
-    <t>CAMISA INSPECTOR BLANCA TALLE 40</t>
-  </si>
-  <si>
-    <t>CAMISA INSPECTOR BLANCA TALLE 42</t>
-  </si>
-  <si>
-    <t>CAMISA INSPECTOR BLANCA TALLE 44</t>
-  </si>
-  <si>
-    <t>CAMISA INSPECTOR BLANCA TALLE 46</t>
-  </si>
-  <si>
-    <t>CAMISA INSPECTOR BLANCA TALLE 48</t>
-  </si>
-  <si>
-    <t>CAMISA INSPECTOR BLANCA TALLE 50</t>
-  </si>
-  <si>
-    <t>CAMISA INSPECTOR BLANCA TALLE 52</t>
-  </si>
-  <si>
-    <t>CAMISA INSPECTOR BLANCA TALLE 58</t>
-  </si>
-  <si>
-    <t>CAMISA INSPECTOR BLANCA TALLE 60</t>
-  </si>
-  <si>
-    <t>CAMISA INSPECTOR BLANCA TALLE 62</t>
-  </si>
-  <si>
-    <t>CAMISA CHOFER MUJER CELESTE TALLE 38</t>
-  </si>
-  <si>
-    <t>CAMISA CHOFER MUJER CELESTE TALLE 40</t>
-  </si>
-  <si>
-    <t>CAMISA CHOFER MUJER CELESTE TALLE 42</t>
-  </si>
-  <si>
-    <t>CAMISA CHOFER MUJER CELESTE TALLE 44</t>
-  </si>
-  <si>
-    <t>CHALECO POLAR NEGRO TALLE M</t>
-  </si>
-  <si>
-    <t>CHALECO POLAR NEGRO TALLE L</t>
-  </si>
-  <si>
-    <t>CHALECO POLAR NEGRO TALLE XL</t>
-  </si>
-  <si>
-    <t>CHALECO POLAR NEGRO TALLE XXL</t>
-  </si>
-  <si>
-    <t>CHALECO POLAR NEGRO TALLE XXXL</t>
-  </si>
-  <si>
-    <t>CHALECO POLAR NEGRO TALLE 4XL</t>
-  </si>
-  <si>
-    <t>CHALECO POLAR NEGRO TALLE 5XL</t>
-  </si>
-  <si>
-    <t>CHALECO POLAR NEGRO TALLE 6XL</t>
-  </si>
-  <si>
-    <t>CAMPERA INSPECCION NEGRA TALLE M</t>
-  </si>
-  <si>
-    <t>CAMPERA INSPECCION NEGRA TALLE L</t>
-  </si>
-  <si>
-    <t>CAMPERA INSPECCION NEGRA TALLE XL</t>
-  </si>
-  <si>
-    <t>CAMPERA INSPECCION NEGRA TALLE XXL</t>
-  </si>
-  <si>
-    <t>CAMPERA INSPECCION NEGRA TALLE XXXL</t>
-  </si>
-  <si>
-    <t>CAMPERA INSPECCION NEGRA TALLE 4XL</t>
-  </si>
-  <si>
-    <t>CAMPERA INSPECCION NEGRA TALLE 5XL</t>
-  </si>
-  <si>
-    <t>CAMPERA INSPECCION NEGRA TALLE 6XL</t>
-  </si>
-  <si>
-    <t>CAMPERA CHOFER AZUL TALLE M</t>
-  </si>
-  <si>
-    <t>CAMPERA CHOFER AZUL TALLE L</t>
-  </si>
-  <si>
-    <t>CAMPERA CHOFER AZUL TALLE XL</t>
-  </si>
-  <si>
-    <t>CAMPERA CHOFER AZUL TALLE XXL</t>
-  </si>
-  <si>
-    <t>CAMPERA CHOFER AZUL TALLE XXXL</t>
-  </si>
-  <si>
-    <t>CAMPERA CHOFER AZUL TALLE 4XL</t>
-  </si>
-  <si>
-    <t>CAMPERA CHOFER AZUL TALLE 5XL</t>
-  </si>
-  <si>
-    <t>CAMPERA CHOFER AZUL TALLE 6XL</t>
-  </si>
-  <si>
-    <t>CAMPERA CHOFER AZUL TALLE 7XL</t>
-  </si>
-  <si>
     <t>FLAVIO</t>
   </si>
   <si>
@@ -388,6 +394,9 @@
     <t>130.00009</t>
   </si>
   <si>
+    <t>130.00010</t>
+  </si>
+  <si>
     <t>130.00011</t>
   </si>
   <si>
@@ -412,6 +421,9 @@
     <t>130.00019</t>
   </si>
   <si>
+    <t>130.00020</t>
+  </si>
+  <si>
     <t>130.00021</t>
   </si>
   <si>
@@ -442,15 +454,27 @@
     <t>130.00044</t>
   </si>
   <si>
+    <t>130.00050</t>
+  </si>
+  <si>
     <t>130.00051</t>
   </si>
   <si>
     <t>130.00057</t>
   </si>
   <si>
+    <t>130.00058</t>
+  </si>
+  <si>
     <t>130.00059</t>
   </si>
   <si>
+    <t>130.00060</t>
+  </si>
+  <si>
+    <t>130.00061</t>
+  </si>
+  <si>
     <t>130.00062</t>
   </si>
   <si>
@@ -475,6 +499,9 @@
     <t>130.00079</t>
   </si>
   <si>
+    <t>130.00080</t>
+  </si>
+  <si>
     <t>130.00081</t>
   </si>
   <si>
@@ -520,6 +547,9 @@
     <t>130.00209</t>
   </si>
   <si>
+    <t>130.00210</t>
+  </si>
+  <si>
     <t>130.00211</t>
   </si>
   <si>
@@ -556,6 +586,9 @@
     <t>130.00229</t>
   </si>
   <si>
+    <t>130.00230</t>
+  </si>
+  <si>
     <t>130.00232</t>
   </si>
   <si>
@@ -577,6 +610,9 @@
     <t>130.00255</t>
   </si>
   <si>
+    <t>130.00260</t>
+  </si>
+  <si>
     <t>130.00261</t>
   </si>
   <si>
@@ -601,6 +637,9 @@
     <t>130.00268</t>
   </si>
   <si>
+    <t>130.00270</t>
+  </si>
+  <si>
     <t>130.00271</t>
   </si>
   <si>
@@ -625,6 +664,9 @@
     <t>130.00278</t>
   </si>
   <si>
+    <t>130.00280</t>
+  </si>
+  <si>
     <t>130.00281</t>
   </si>
   <si>
@@ -650,6 +692,9 @@
   </si>
   <si>
     <t>130.00289</t>
+  </si>
+  <si>
+    <t>130.00290</t>
   </si>
 </sst>
 </file>
@@ -981,7 +1026,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F109"/>
+  <dimension ref="A1:F111"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1009,7 +1054,7 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D2">
         <v>130</v>
@@ -1018,7 +1063,7 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1029,16 +1074,16 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D3">
         <v>130</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1049,16 +1094,16 @@
         <v>7</v>
       </c>
       <c r="C4" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D4">
         <v>130</v>
       </c>
       <c r="E4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F4" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1069,16 +1114,16 @@
         <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D5">
         <v>130</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F5" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1089,16 +1134,16 @@
         <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D6">
         <v>130</v>
       </c>
       <c r="E6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F6" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1109,16 +1154,16 @@
         <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D7">
         <v>130</v>
       </c>
       <c r="E7">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1129,16 +1174,16 @@
         <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D8">
         <v>130</v>
       </c>
       <c r="E8">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F8" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1149,16 +1194,16 @@
         <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D9">
         <v>130</v>
       </c>
       <c r="E9">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F9" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1169,16 +1214,16 @@
         <v>13</v>
       </c>
       <c r="C10" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D10">
         <v>130</v>
       </c>
       <c r="E10">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F10" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1189,16 +1234,16 @@
         <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D11">
         <v>130</v>
       </c>
       <c r="E11">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1209,16 +1254,16 @@
         <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D12">
         <v>130</v>
       </c>
       <c r="E12">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F12" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1229,16 +1274,16 @@
         <v>16</v>
       </c>
       <c r="C13" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D13">
         <v>130</v>
       </c>
       <c r="E13">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F13" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1249,16 +1294,16 @@
         <v>17</v>
       </c>
       <c r="C14" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D14">
         <v>130</v>
       </c>
       <c r="E14">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F14" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -1269,16 +1314,16 @@
         <v>18</v>
       </c>
       <c r="C15" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D15">
         <v>130</v>
       </c>
       <c r="E15">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="F15" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1289,16 +1334,16 @@
         <v>19</v>
       </c>
       <c r="C16" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D16">
         <v>130</v>
       </c>
       <c r="E16">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F16" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1309,16 +1354,16 @@
         <v>20</v>
       </c>
       <c r="C17" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D17">
         <v>130</v>
       </c>
       <c r="E17">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F17" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1329,16 +1374,16 @@
         <v>21</v>
       </c>
       <c r="C18" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D18">
         <v>130</v>
       </c>
       <c r="E18">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F18" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -1349,16 +1394,16 @@
         <v>22</v>
       </c>
       <c r="C19" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D19">
         <v>130</v>
       </c>
       <c r="E19">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F19" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -1369,16 +1414,16 @@
         <v>23</v>
       </c>
       <c r="C20" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D20">
         <v>130</v>
       </c>
       <c r="E20">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F20" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -1389,16 +1434,16 @@
         <v>24</v>
       </c>
       <c r="C21" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D21">
         <v>130</v>
       </c>
       <c r="E21">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F21" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -1409,16 +1454,16 @@
         <v>25</v>
       </c>
       <c r="C22" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D22">
         <v>130</v>
       </c>
       <c r="E22">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F22" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -1429,16 +1474,16 @@
         <v>26</v>
       </c>
       <c r="C23" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D23">
         <v>130</v>
       </c>
       <c r="E23">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F23" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -1449,16 +1494,16 @@
         <v>27</v>
       </c>
       <c r="C24" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D24">
         <v>130</v>
       </c>
       <c r="E24">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F24" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -1469,16 +1514,16 @@
         <v>28</v>
       </c>
       <c r="C25" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D25">
         <v>130</v>
       </c>
       <c r="E25">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F25" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -1489,16 +1534,16 @@
         <v>29</v>
       </c>
       <c r="C26" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D26">
         <v>130</v>
       </c>
       <c r="E26">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F26" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -1509,16 +1554,16 @@
         <v>30</v>
       </c>
       <c r="C27" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D27">
         <v>130</v>
       </c>
       <c r="E27">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F27" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -1529,16 +1574,16 @@
         <v>31</v>
       </c>
       <c r="C28" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D28">
         <v>130</v>
       </c>
       <c r="E28">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F28" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -1549,16 +1594,16 @@
         <v>32</v>
       </c>
       <c r="C29" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D29">
         <v>130</v>
       </c>
       <c r="E29">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F29" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -1569,16 +1614,16 @@
         <v>33</v>
       </c>
       <c r="C30" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D30">
         <v>130</v>
       </c>
       <c r="E30">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="F30" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -1589,16 +1634,16 @@
         <v>34</v>
       </c>
       <c r="C31" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D31">
         <v>130</v>
       </c>
       <c r="E31">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="F31" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -1609,16 +1654,16 @@
         <v>35</v>
       </c>
       <c r="C32" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D32">
         <v>130</v>
       </c>
       <c r="E32">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="F32" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -1629,16 +1674,16 @@
         <v>36</v>
       </c>
       <c r="C33" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D33">
         <v>130</v>
       </c>
       <c r="E33">
-        <v>27</v>
+        <v>57</v>
       </c>
       <c r="F33" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -1649,16 +1694,16 @@
         <v>37</v>
       </c>
       <c r="C34" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D34">
         <v>130</v>
       </c>
       <c r="E34">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="F34" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -1669,16 +1714,16 @@
         <v>38</v>
       </c>
       <c r="C35" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D35">
         <v>130</v>
       </c>
       <c r="E35">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="F35" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -1689,16 +1734,16 @@
         <v>39</v>
       </c>
       <c r="C36" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D36">
         <v>130</v>
       </c>
       <c r="E36">
-        <v>28</v>
+        <v>60</v>
       </c>
       <c r="F36" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -1709,16 +1754,16 @@
         <v>40</v>
       </c>
       <c r="C37" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D37">
         <v>130</v>
       </c>
       <c r="E37">
-        <v>29</v>
+        <v>61</v>
       </c>
       <c r="F37" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -1729,16 +1774,16 @@
         <v>41</v>
       </c>
       <c r="C38" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D38">
         <v>130</v>
       </c>
       <c r="E38">
-        <v>29</v>
+        <v>62</v>
       </c>
       <c r="F38" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -1749,16 +1794,16 @@
         <v>42</v>
       </c>
       <c r="C39" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D39">
         <v>130</v>
       </c>
       <c r="E39">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="F39" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -1769,16 +1814,16 @@
         <v>43</v>
       </c>
       <c r="C40" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D40">
         <v>130</v>
       </c>
       <c r="E40">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="F40" t="s">
-        <v>142</v>
+        <v>155</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -1789,16 +1834,16 @@
         <v>44</v>
       </c>
       <c r="C41" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D41">
         <v>130</v>
       </c>
       <c r="E41">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="F41" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -1809,16 +1854,16 @@
         <v>45</v>
       </c>
       <c r="C42" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D42">
         <v>130</v>
       </c>
       <c r="E42">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="F42" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -1829,16 +1874,16 @@
         <v>46</v>
       </c>
       <c r="C43" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D43">
         <v>130</v>
       </c>
       <c r="E43">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="F43" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -1849,16 +1894,16 @@
         <v>47</v>
       </c>
       <c r="C44" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D44">
         <v>130</v>
       </c>
       <c r="E44">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="F44" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
     </row>
     <row r="45" spans="1:6">
@@ -1869,16 +1914,16 @@
         <v>48</v>
       </c>
       <c r="C45" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D45">
         <v>130</v>
       </c>
       <c r="E45">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="F45" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
     </row>
     <row r="46" spans="1:6">
@@ -1889,16 +1934,16 @@
         <v>49</v>
       </c>
       <c r="C46" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D46">
         <v>130</v>
       </c>
       <c r="E46">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="F46" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
     </row>
     <row r="47" spans="1:6">
@@ -1909,16 +1954,16 @@
         <v>50</v>
       </c>
       <c r="C47" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D47">
         <v>130</v>
       </c>
       <c r="E47">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F47" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
     </row>
     <row r="48" spans="1:6">
@@ -1929,16 +1974,16 @@
         <v>51</v>
       </c>
       <c r="C48" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D48">
         <v>130</v>
       </c>
       <c r="E48">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="F48" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
     </row>
     <row r="49" spans="1:6">
@@ -1949,16 +1994,16 @@
         <v>52</v>
       </c>
       <c r="C49" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D49">
         <v>130</v>
       </c>
       <c r="E49">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="F49" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
     </row>
     <row r="50" spans="1:6">
@@ -1969,16 +2014,16 @@
         <v>53</v>
       </c>
       <c r="C50" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D50">
         <v>130</v>
       </c>
       <c r="E50">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="F50" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
     </row>
     <row r="51" spans="1:6">
@@ -1989,16 +2034,16 @@
         <v>54</v>
       </c>
       <c r="C51" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D51">
         <v>130</v>
       </c>
       <c r="E51">
-        <v>81</v>
+        <v>122</v>
       </c>
       <c r="F51" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
     </row>
     <row r="52" spans="1:6">
@@ -2009,16 +2054,16 @@
         <v>55</v>
       </c>
       <c r="C52" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D52">
         <v>130</v>
       </c>
       <c r="E52">
-        <v>82</v>
+        <v>125</v>
       </c>
       <c r="F52" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
     </row>
     <row r="53" spans="1:6">
@@ -2029,16 +2074,16 @@
         <v>56</v>
       </c>
       <c r="C53" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D53">
         <v>130</v>
       </c>
       <c r="E53">
-        <v>85</v>
+        <v>201</v>
       </c>
       <c r="F53" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
     </row>
     <row r="54" spans="1:6">
@@ -2049,16 +2094,16 @@
         <v>57</v>
       </c>
       <c r="C54" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D54">
         <v>130</v>
       </c>
       <c r="E54">
-        <v>88</v>
+        <v>202</v>
       </c>
       <c r="F54" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
     </row>
     <row r="55" spans="1:6">
@@ -2069,16 +2114,16 @@
         <v>58</v>
       </c>
       <c r="C55" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D55">
         <v>130</v>
       </c>
       <c r="E55">
-        <v>122</v>
+        <v>203</v>
       </c>
       <c r="F55" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
     </row>
     <row r="56" spans="1:6">
@@ -2089,16 +2134,16 @@
         <v>59</v>
       </c>
       <c r="C56" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D56">
         <v>130</v>
       </c>
       <c r="E56">
-        <v>125</v>
+        <v>204</v>
       </c>
       <c r="F56" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
     </row>
     <row r="57" spans="1:6">
@@ -2109,16 +2154,16 @@
         <v>60</v>
       </c>
       <c r="C57" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D57">
         <v>130</v>
       </c>
       <c r="E57">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="F57" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
     </row>
     <row r="58" spans="1:6">
@@ -2129,16 +2174,16 @@
         <v>61</v>
       </c>
       <c r="C58" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D58">
         <v>130</v>
       </c>
       <c r="E58">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="F58" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
     </row>
     <row r="59" spans="1:6">
@@ -2149,16 +2194,16 @@
         <v>62</v>
       </c>
       <c r="C59" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D59">
         <v>130</v>
       </c>
       <c r="E59">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="F59" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -2169,16 +2214,16 @@
         <v>63</v>
       </c>
       <c r="C60" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D60">
         <v>130</v>
       </c>
       <c r="E60">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="F60" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
     </row>
     <row r="61" spans="1:6">
@@ -2189,16 +2234,16 @@
         <v>64</v>
       </c>
       <c r="C61" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D61">
         <v>130</v>
       </c>
       <c r="E61">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="F61" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
     </row>
     <row r="62" spans="1:6">
@@ -2209,16 +2254,16 @@
         <v>65</v>
       </c>
       <c r="C62" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D62">
         <v>130</v>
       </c>
       <c r="E62">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="F62" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
     </row>
     <row r="63" spans="1:6">
@@ -2229,16 +2274,16 @@
         <v>66</v>
       </c>
       <c r="C63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D63">
         <v>130</v>
       </c>
       <c r="E63">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="F63" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
     </row>
     <row r="64" spans="1:6">
@@ -2249,16 +2294,16 @@
         <v>67</v>
       </c>
       <c r="C64" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D64">
         <v>130</v>
       </c>
       <c r="E64">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="F64" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
     </row>
     <row r="65" spans="1:6">
@@ -2269,16 +2314,16 @@
         <v>68</v>
       </c>
       <c r="C65" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D65">
         <v>130</v>
       </c>
       <c r="E65">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="F65" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
     </row>
     <row r="66" spans="1:6">
@@ -2289,16 +2334,16 @@
         <v>69</v>
       </c>
       <c r="C66" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D66">
         <v>130</v>
       </c>
       <c r="E66">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="F66" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
     </row>
     <row r="67" spans="1:6">
@@ -2309,16 +2354,16 @@
         <v>70</v>
       </c>
       <c r="C67" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D67">
         <v>130</v>
       </c>
       <c r="E67">
-        <v>212</v>
+        <v>222</v>
       </c>
       <c r="F67" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
     </row>
     <row r="68" spans="1:6">
@@ -2329,16 +2374,16 @@
         <v>71</v>
       </c>
       <c r="C68" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D68">
         <v>130</v>
       </c>
       <c r="E68">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="F68" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
     </row>
     <row r="69" spans="1:6">
@@ -2349,16 +2394,16 @@
         <v>72</v>
       </c>
       <c r="C69" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D69">
         <v>130</v>
       </c>
       <c r="E69">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="F69" t="s">
-        <v>171</v>
+        <v>184</v>
       </c>
     </row>
     <row r="70" spans="1:6">
@@ -2369,16 +2414,16 @@
         <v>73</v>
       </c>
       <c r="C70" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D70">
         <v>130</v>
       </c>
       <c r="E70">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="F70" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
     </row>
     <row r="71" spans="1:6">
@@ -2389,16 +2434,16 @@
         <v>74</v>
       </c>
       <c r="C71" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D71">
         <v>130</v>
       </c>
       <c r="E71">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="F71" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
     </row>
     <row r="72" spans="1:6">
@@ -2409,16 +2454,16 @@
         <v>75</v>
       </c>
       <c r="C72" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D72">
         <v>130</v>
       </c>
       <c r="E72">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="F72" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
     </row>
     <row r="73" spans="1:6">
@@ -2429,16 +2474,16 @@
         <v>76</v>
       </c>
       <c r="C73" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D73">
         <v>130</v>
       </c>
       <c r="E73">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="F73" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
     </row>
     <row r="74" spans="1:6">
@@ -2449,16 +2494,16 @@
         <v>77</v>
       </c>
       <c r="C74" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D74">
         <v>130</v>
       </c>
       <c r="E74">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="F74" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
     </row>
     <row r="75" spans="1:6">
@@ -2469,16 +2514,16 @@
         <v>78</v>
       </c>
       <c r="C75" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D75">
         <v>130</v>
       </c>
       <c r="E75">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="F75" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
     </row>
     <row r="76" spans="1:6">
@@ -2489,16 +2534,16 @@
         <v>79</v>
       </c>
       <c r="C76" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D76">
         <v>130</v>
       </c>
       <c r="E76">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="F76" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
     </row>
     <row r="77" spans="1:6">
@@ -2509,16 +2554,16 @@
         <v>80</v>
       </c>
       <c r="C77" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D77">
         <v>130</v>
       </c>
       <c r="E77">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="F77" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
     </row>
     <row r="78" spans="1:6">
@@ -2529,16 +2574,16 @@
         <v>81</v>
       </c>
       <c r="C78" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D78">
         <v>130</v>
       </c>
       <c r="E78">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="F78" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
     </row>
     <row r="79" spans="1:6">
@@ -2549,16 +2594,16 @@
         <v>82</v>
       </c>
       <c r="C79" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D79">
         <v>130</v>
       </c>
       <c r="E79">
-        <v>233</v>
+        <v>252</v>
       </c>
       <c r="F79" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
     </row>
     <row r="80" spans="1:6">
@@ -2569,16 +2614,16 @@
         <v>83</v>
       </c>
       <c r="C80" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D80">
         <v>130</v>
       </c>
       <c r="E80">
-        <v>234</v>
+        <v>253</v>
       </c>
       <c r="F80" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
     </row>
     <row r="81" spans="1:6">
@@ -2589,16 +2634,16 @@
         <v>84</v>
       </c>
       <c r="C81" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D81">
         <v>130</v>
       </c>
       <c r="E81">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="F81" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
     </row>
     <row r="82" spans="1:6">
@@ -2609,16 +2654,16 @@
         <v>85</v>
       </c>
       <c r="C82" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D82">
         <v>130</v>
       </c>
       <c r="E82">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="F82" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
     </row>
     <row r="83" spans="1:6">
@@ -2629,16 +2674,16 @@
         <v>86</v>
       </c>
       <c r="C83" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D83">
         <v>130</v>
       </c>
       <c r="E83">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="F83" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
     </row>
     <row r="84" spans="1:6">
@@ -2649,16 +2694,16 @@
         <v>87</v>
       </c>
       <c r="C84" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D84">
         <v>130</v>
       </c>
       <c r="E84">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="F84" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
     </row>
     <row r="85" spans="1:6">
@@ -2669,16 +2714,16 @@
         <v>88</v>
       </c>
       <c r="C85" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D85">
         <v>130</v>
       </c>
       <c r="E85">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F85" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
     </row>
     <row r="86" spans="1:6">
@@ -2689,16 +2734,16 @@
         <v>89</v>
       </c>
       <c r="C86" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D86">
         <v>130</v>
       </c>
       <c r="E86">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F86" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
     </row>
     <row r="87" spans="1:6">
@@ -2709,16 +2754,16 @@
         <v>90</v>
       </c>
       <c r="C87" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D87">
         <v>130</v>
       </c>
       <c r="E87">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F87" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
     </row>
     <row r="88" spans="1:6">
@@ -2729,16 +2774,16 @@
         <v>91</v>
       </c>
       <c r="C88" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D88">
         <v>130</v>
       </c>
       <c r="E88">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F88" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
     </row>
     <row r="89" spans="1:6">
@@ -2749,16 +2794,16 @@
         <v>92</v>
       </c>
       <c r="C89" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D89">
         <v>130</v>
       </c>
       <c r="E89">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="F89" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
     </row>
     <row r="90" spans="1:6">
@@ -2769,16 +2814,16 @@
         <v>93</v>
       </c>
       <c r="C90" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D90">
         <v>130</v>
       </c>
       <c r="E90">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F90" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
     </row>
     <row r="91" spans="1:6">
@@ -2789,16 +2834,16 @@
         <v>94</v>
       </c>
       <c r="C91" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D91">
         <v>130</v>
       </c>
       <c r="E91">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F91" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
     </row>
     <row r="92" spans="1:6">
@@ -2809,16 +2854,16 @@
         <v>95</v>
       </c>
       <c r="C92" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D92">
         <v>130</v>
       </c>
       <c r="E92">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="F92" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
     </row>
     <row r="93" spans="1:6">
@@ -2829,7 +2874,7 @@
         <v>96</v>
       </c>
       <c r="C93" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D93">
         <v>130</v>
@@ -2838,7 +2883,7 @@
         <v>271</v>
       </c>
       <c r="F93" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
     </row>
     <row r="94" spans="1:6">
@@ -2849,7 +2894,7 @@
         <v>97</v>
       </c>
       <c r="C94" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D94">
         <v>130</v>
@@ -2858,7 +2903,7 @@
         <v>272</v>
       </c>
       <c r="F94" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
     </row>
     <row r="95" spans="1:6">
@@ -2869,7 +2914,7 @@
         <v>98</v>
       </c>
       <c r="C95" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D95">
         <v>130</v>
@@ -2878,7 +2923,7 @@
         <v>273</v>
       </c>
       <c r="F95" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
     </row>
     <row r="96" spans="1:6">
@@ -2889,7 +2934,7 @@
         <v>99</v>
       </c>
       <c r="C96" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D96">
         <v>130</v>
@@ -2898,7 +2943,7 @@
         <v>274</v>
       </c>
       <c r="F96" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
     </row>
     <row r="97" spans="1:6">
@@ -2909,7 +2954,7 @@
         <v>100</v>
       </c>
       <c r="C97" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D97">
         <v>130</v>
@@ -2918,7 +2963,7 @@
         <v>275</v>
       </c>
       <c r="F97" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
     </row>
     <row r="98" spans="1:6">
@@ -2929,7 +2974,7 @@
         <v>101</v>
       </c>
       <c r="C98" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D98">
         <v>130</v>
@@ -2938,7 +2983,7 @@
         <v>276</v>
       </c>
       <c r="F98" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
     </row>
     <row r="99" spans="1:6">
@@ -2949,7 +2994,7 @@
         <v>102</v>
       </c>
       <c r="C99" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D99">
         <v>130</v>
@@ -2958,7 +3003,7 @@
         <v>277</v>
       </c>
       <c r="F99" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
     </row>
     <row r="100" spans="1:6">
@@ -2969,7 +3014,7 @@
         <v>103</v>
       </c>
       <c r="C100" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D100">
         <v>130</v>
@@ -2978,7 +3023,7 @@
         <v>278</v>
       </c>
       <c r="F100" t="s">
-        <v>202</v>
+        <v>215</v>
       </c>
     </row>
     <row r="101" spans="1:6">
@@ -2989,16 +3034,16 @@
         <v>104</v>
       </c>
       <c r="C101" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D101">
         <v>130</v>
       </c>
       <c r="E101">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F101" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
     </row>
     <row r="102" spans="1:6">
@@ -3009,16 +3054,16 @@
         <v>105</v>
       </c>
       <c r="C102" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D102">
         <v>130</v>
       </c>
       <c r="E102">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F102" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
     </row>
     <row r="103" spans="1:6">
@@ -3029,16 +3074,16 @@
         <v>106</v>
       </c>
       <c r="C103" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D103">
         <v>130</v>
       </c>
       <c r="E103">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F103" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
     </row>
     <row r="104" spans="1:6">
@@ -3049,16 +3094,16 @@
         <v>107</v>
       </c>
       <c r="C104" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D104">
         <v>130</v>
       </c>
       <c r="E104">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F104" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
     </row>
     <row r="105" spans="1:6">
@@ -3069,16 +3114,16 @@
         <v>108</v>
       </c>
       <c r="C105" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D105">
         <v>130</v>
       </c>
       <c r="E105">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F105" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
     </row>
     <row r="106" spans="1:6">
@@ -3089,16 +3134,16 @@
         <v>109</v>
       </c>
       <c r="C106" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D106">
         <v>130</v>
       </c>
       <c r="E106">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F106" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
     </row>
     <row r="107" spans="1:6">
@@ -3109,16 +3154,16 @@
         <v>110</v>
       </c>
       <c r="C107" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D107">
         <v>130</v>
       </c>
       <c r="E107">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F107" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
     </row>
     <row r="108" spans="1:6">
@@ -3129,16 +3174,16 @@
         <v>111</v>
       </c>
       <c r="C108" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D108">
         <v>130</v>
       </c>
       <c r="E108">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="F108" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
     </row>
     <row r="109" spans="1:6">
@@ -3149,16 +3194,56 @@
         <v>112</v>
       </c>
       <c r="C109" t="s">
+        <v>115</v>
+      </c>
+      <c r="D109">
+        <v>130</v>
+      </c>
+      <c r="E109">
+        <v>288</v>
+      </c>
+      <c r="F109" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6">
+      <c r="A110">
+        <v>108</v>
+      </c>
+      <c r="B110" t="s">
         <v>113</v>
       </c>
-      <c r="D109">
-        <v>130</v>
-      </c>
-      <c r="E109">
+      <c r="C110" t="s">
+        <v>115</v>
+      </c>
+      <c r="D110">
+        <v>130</v>
+      </c>
+      <c r="E110">
         <v>289</v>
       </c>
-      <c r="F109" t="s">
-        <v>211</v>
+      <c r="F110" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6">
+      <c r="A111">
+        <v>109</v>
+      </c>
+      <c r="B111" t="s">
+        <v>114</v>
+      </c>
+      <c r="C111" t="s">
+        <v>115</v>
+      </c>
+      <c r="D111">
+        <v>130</v>
+      </c>
+      <c r="E111">
+        <v>290</v>
+      </c>
+      <c r="F111" t="s">
+        <v>226</v>
       </c>
     </row>
   </sheetData>

</xml_diff>